<commit_message>
Fixed bug with custom_field_headers in all imports
</commit_message>
<xml_diff>
--- a/public/sample_uploads/portfolio_investments.xlsx
+++ b/public/sample_uploads/portfolio_investments.xlsx
@@ -195,7 +195,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="22">
   <si>
     <t xml:space="preserve">Fund</t>
   </si>
@@ -228,6 +228,9 @@
   </si>
   <si>
     <t xml:space="preserve">Proforma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ref Id</t>
   </si>
   <si>
     <t xml:space="preserve">SAAS Fund</t>
@@ -617,7 +620,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultColWidth="8.53515625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.26"/>
@@ -671,13 +674,16 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>43831</v>
@@ -689,24 +695,27 @@
         <v>20000</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>44197</v>
@@ -718,24 +727,27 @@
         <v>12000</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>44562</v>
@@ -747,24 +759,27 @@
         <v>-20000</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>43831</v>
@@ -776,24 +791,27 @@
         <v>10000</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>44927</v>
@@ -805,24 +823,27 @@
         <v>-3000</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>44228</v>
@@ -834,24 +855,27 @@
         <v>12000</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>43831</v>
@@ -863,24 +887,27 @@
         <v>20000</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L8" s="1" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>43831</v>
@@ -892,24 +919,27 @@
         <v>-10000</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>43832</v>
@@ -921,19 +951,22 @@
         <v>30000</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>